<commit_message>
Update price, config and deal data
</commit_message>
<xml_diff>
--- a/config_sets.xlsx
+++ b/config_sets.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,11 +496,7 @@
           <t>1872</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>https://www.lego.com/cdn/cs/set/assets/blt55fbccadb7d66885/10300.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
@@ -764,11 +760,7 @@
           <t>806</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>https://www.lego.com/cdn/cs/set/assets/bltb82764353d6cd9c2/bltaa6c5faaf18aa138-11505_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
@@ -832,11 +824,7 @@
           <t>2193</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>https://www.lego.com/cdn/cs/set/assets/blta1405340d716cd20/21351_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
@@ -919,28 +907,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>45200</t>
+          <t>42232</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kit de science Mission lunaire</t>
+          <t>Megacar Sadair's Spear de Koenigsegg</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>519</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>4104</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltf7b7ce8f03c1660e/bltb54bf9af8b6f95a9-45200_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltdd490f7023a9625c/blt115568a63fa37862-42232_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/45200</t>
+          <t>https://www.lego.com/fr-fr/product/42232</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -951,32 +943,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>45201</t>
+          <t>45200</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Kit de science Animaux de l’Antarctique</t>
+          <t>Kit de science Mission lunaire</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>461</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+          <t>519</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/blte5a2e0694b4165e5/blt4370f603aae1af0d-45201_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltf7b7ce8f03c1660e/bltb54bf9af8b6f95a9-45200_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/45201</t>
+          <t>https://www.lego.com/fr-fr/product/45200</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -987,32 +975,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>80121</t>
+          <t>45201</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>L’auberge traditionnelle du clair de lune</t>
+          <t>Kit de science Animaux de l’Antarctique</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1530</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+          <t>461</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://www.lego.com/cdn/cs/set/assets/bltfc4f59188fa9bf87/blt00132fa0deebd2ee-80121_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+          <t>https://www.lego.com/cdn/cs/set/assets/blte5a2e0694b4165e5/blt4370f603aae1af0d-45201_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.lego.com/fr-fr/product/80121</t>
+          <t>https://www.lego.com/fr-fr/product/45201</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1020,6 +1004,38 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>80121</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>L’auberge traditionnelle du clair de lune</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://www.lego.com/cdn/cs/set/assets/bltfc4f59188fa9bf87/blt00132fa0deebd2ee-80121_Prod.png?format=webply&amp;fit=bounds&amp;quality=75&amp;width=528&amp;height=528&amp;dpr=1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://www.lego.com/fr-fr/product/80121</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>